<commit_message>
updates to docs/proc compare parity
</commit_message>
<xml_diff>
--- a/inst/out/compare-report-roster-2021-2022.xlsx
+++ b/inst/out/compare-report-roster-2021-2022.xlsx
@@ -12,12 +12,15 @@
     <sheet name="Review Changes" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Base Data" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Compare Data" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Column Diffs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Class Diffs" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Summary" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="583">
   <si>
     <t xml:space="preserve">subject_id</t>
   </si>
@@ -1709,6 +1712,63 @@
   </si>
   <si>
     <t xml:space="preserve">Avery Lopez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class_base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class_compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_new</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_deleted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_vars_base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_vars_compare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_vars_common</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_vars_base_only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_vars_compare_only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_vars_with_diffs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_value_diffs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_class_mismatches</t>
   </si>
 </sst>
 </file>
@@ -19144,4 +19204,256 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>564</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>565</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>564</v>
+      </c>
+      <c r="B1" t="s">
+        <v>566</v>
+      </c>
+      <c r="C1" t="s">
+        <v>567</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>568</v>
+      </c>
+      <c r="B1" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B2" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>571</v>
+      </c>
+      <c r="B3" t="n">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>572</v>
+      </c>
+      <c r="B4" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>573</v>
+      </c>
+      <c r="B5" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>574</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>575</v>
+      </c>
+      <c r="B7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>576</v>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>577</v>
+      </c>
+      <c r="B9" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>578</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>579</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>580</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>581</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>582</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>